<commit_message>
Updates to general ID code. Force generation of certain IDs that do not need calculating to properly format the IDs
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/pha4ge-to-v2/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/pha4ge-to-v2/ids/general_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/pha4ge-to-v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C3674E2-3DA5-1A4E-B1CE-F77060E1521E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44239EFA-4079-8540-8AD6-0DDF92032300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="94">
   <si>
     <t>addresses</t>
   </si>
@@ -314,6 +314,9 @@
   </si>
   <si>
     <t>fn.makeid(dat.protocols.__protocolID)</t>
+  </si>
+  <si>
+    <t>datEmpty.organizations.organizationID</t>
   </si>
 </sst>
 </file>
@@ -785,7 +788,7 @@
         <v>87</v>
       </c>
       <c r="D12" t="s">
-        <v>47</v>
+        <v>93</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added measureSets, more linkage paths, and additional ID generation changes
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/pha4ge-to-v2/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/pha4ge-to-v2/ids/general_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/pha4ge-to-v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44239EFA-4079-8540-8AD6-0DDF92032300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF58A7AE-83FE-0043-B45F-3004336A94C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="95">
   <si>
     <t>addresses</t>
   </si>
@@ -259,9 +259,6 @@
     <t>fn.makeid(datEmpty.samples.siteID, datEmpty.samples.collDT if dat.samples.collDT else datEmpty.samples.collDTEnd, f"{fn.rownum:03d}")</t>
   </si>
   <si>
-    <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(fn.countrows("measures", "(__source_file_and_row__)", equals=dat.measureSets.get("(__source_file_and_row__)"))))</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.addresses.country, datEmpty.addresses.pCode, datEmpty.addresses.city[:3])</t>
   </si>
   <si>
@@ -317,6 +314,12 @@
   </si>
   <si>
     <t>datEmpty.organizations.organizationID</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(fn.countrows("measures")))</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.qualityReports.qualityFlag, dat.qualityReports.measureRepID, dat.qualityReports.sampleID, dat.qualityReports.measureSetRepID)</t>
   </si>
 </sst>
 </file>
@@ -360,9 +363,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -708,10 +712,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E2" t="s">
         <v>67</v>
@@ -736,7 +740,7 @@
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D5" t="s">
         <v>59</v>
@@ -785,10 +789,10 @@
         <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -831,7 +835,7 @@
         <v>16</v>
       </c>
       <c r="C18" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D18" t="s">
         <v>60</v>
@@ -886,7 +890,7 @@
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D25" t="s">
         <v>61</v>
@@ -990,8 +994,8 @@
       <c r="B35" t="s">
         <v>9</v>
       </c>
-      <c r="C35" t="s">
-        <v>74</v>
+      <c r="C35" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="E35" t="s">
         <v>62</v>
@@ -1038,7 +1042,7 @@
         <v>10</v>
       </c>
       <c r="C40" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D40" t="s">
         <v>63</v>
@@ -1074,7 +1078,7 @@
         <v>7</v>
       </c>
       <c r="C44" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D44" t="s">
         <v>64</v>
@@ -1121,10 +1125,10 @@
         <v>37</v>
       </c>
       <c r="B49" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C49" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -1143,7 +1147,7 @@
         <v>5</v>
       </c>
       <c r="C52" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D52" t="s">
         <v>65</v>
@@ -1234,6 +1238,9 @@
         <v>18</v>
       </c>
       <c r="C62" t="s">
+        <v>94</v>
+      </c>
+      <c r="E62" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1269,6 +1276,9 @@
       <c r="B65" t="s">
         <v>9</v>
       </c>
+      <c r="C65" t="s">
+        <v>53</v>
+      </c>
       <c r="E65" t="s">
         <v>58</v>
       </c>
@@ -1286,7 +1296,7 @@
         <v>6</v>
       </c>
       <c r="C69" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D69" t="s">
         <v>73</v>
@@ -1355,7 +1365,7 @@
         <v>70</v>
       </c>
       <c r="C75" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
@@ -1363,10 +1373,10 @@
         <v>19</v>
       </c>
       <c r="B76" t="s">
+        <v>78</v>
+      </c>
+      <c r="C76" t="s">
         <v>79</v>
-      </c>
-      <c r="C76" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
@@ -1374,10 +1384,10 @@
         <v>19</v>
       </c>
       <c r="B77" t="s">
+        <v>80</v>
+      </c>
+      <c r="C77" t="s">
         <v>81</v>
-      </c>
-      <c r="C77" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
@@ -1396,7 +1406,7 @@
         <v>8</v>
       </c>
       <c r="C80" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D80" t="s">
         <v>66</v>

</xml_diff>